<commit_message>
fix(shopee): leave brand empty and clean mass upload format for seller centre
</commit_message>
<xml_diff>
--- a/docs/Shopee_mass_upload_FILLED_basic.xlsx
+++ b/docs/Shopee_mass_upload_FILLED_basic.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{750BD9DD-A040-47E1-AC34-B9D8D6D7F0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D4B60A-AF90-48A1-8280-150C1A6160DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5917" uniqueCount="3815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5917" uniqueCount="3814">
   <si>
     <t>Tentang Template Mass Upload</t>
   </si>
@@ -11455,9 +11455,6 @@
   </si>
   <si>
     <t>VND-MSTR-ALL</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>https://raw.githubusercontent.com/adrian-dev-art/vendoraman/main/docs/shopee_assets/cover_master_bundle.jpg</t>
@@ -13332,6 +13329,9 @@
       </c>
     </row>
     <row r="7" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>101514</v>
+      </c>
       <c r="B7" s="2" t="s">
         <v>3784</v>
       </c>
@@ -13342,7 +13342,7 @@
         <v>3786</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q7" s="2">
         <v>149000</v>
@@ -13351,22 +13351,22 @@
         <v>999</v>
       </c>
       <c r="W7" s="2" t="s">
+        <v>3787</v>
+      </c>
+      <c r="X7" s="2" t="s">
         <v>3788</v>
       </c>
-      <c r="X7" s="2" t="s">
+      <c r="Y7" s="2" t="s">
         <v>3789</v>
       </c>
-      <c r="Y7" s="2" t="s">
+      <c r="Z7" s="2" t="s">
         <v>3790</v>
       </c>
-      <c r="Z7" s="2" t="s">
+      <c r="AA7" s="2" t="s">
         <v>3791</v>
       </c>
-      <c r="AA7" s="2" t="s">
+      <c r="AB7" s="2" t="s">
         <v>3792</v>
-      </c>
-      <c r="AB7" s="2" t="s">
-        <v>3793</v>
       </c>
       <c r="AF7" s="2">
         <v>10</v>
@@ -13385,17 +13385,20 @@
       </c>
     </row>
     <row r="8" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>101514</v>
+      </c>
       <c r="B8" s="2" t="s">
+        <v>3793</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>3794</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>3795</v>
       </c>
-      <c r="I8" s="2" t="s">
-        <v>3796</v>
-      </c>
       <c r="J8" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q8" s="2">
         <v>69000</v>
@@ -13404,19 +13407,19 @@
         <v>999</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>3792</v>
+        <v>3791</v>
       </c>
       <c r="X8" s="2" t="s">
+        <v>3788</v>
+      </c>
+      <c r="Y8" s="2" t="s">
         <v>3789</v>
       </c>
-      <c r="Y8" s="2" t="s">
+      <c r="Z8" s="2" t="s">
         <v>3790</v>
       </c>
-      <c r="Z8" s="2" t="s">
-        <v>3791</v>
-      </c>
       <c r="AA8" s="2" t="s">
-        <v>3788</v>
+        <v>3787</v>
       </c>
       <c r="AF8" s="2">
         <v>10</v>
@@ -13435,17 +13438,20 @@
       </c>
     </row>
     <row r="9" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>101514</v>
+      </c>
       <c r="B9" s="2" t="s">
+        <v>3796</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>3797</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>3798</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>3799</v>
-      </c>
       <c r="J9" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q9" s="2">
         <v>59000</v>
@@ -13454,19 +13460,19 @@
         <v>999</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>3793</v>
+        <v>3792</v>
       </c>
       <c r="X9" s="2" t="s">
+        <v>3788</v>
+      </c>
+      <c r="Y9" s="2" t="s">
         <v>3789</v>
       </c>
-      <c r="Y9" s="2" t="s">
+      <c r="Z9" s="2" t="s">
         <v>3790</v>
       </c>
-      <c r="Z9" s="2" t="s">
-        <v>3791</v>
-      </c>
       <c r="AA9" s="2" t="s">
-        <v>3788</v>
+        <v>3787</v>
       </c>
       <c r="AF9" s="2">
         <v>10</v>
@@ -13485,17 +13491,20 @@
       </c>
     </row>
     <row r="10" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>101514</v>
+      </c>
       <c r="B10" s="2" t="s">
+        <v>3799</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>3800</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>3801</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>3802</v>
-      </c>
       <c r="J10" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q10" s="2">
         <v>49000</v>
@@ -13504,16 +13513,16 @@
         <v>999</v>
       </c>
       <c r="W10" s="2" t="s">
+        <v>3787</v>
+      </c>
+      <c r="X10" s="2" t="s">
         <v>3788</v>
       </c>
-      <c r="X10" s="2" t="s">
+      <c r="Y10" s="2" t="s">
         <v>3789</v>
       </c>
-      <c r="Y10" s="2" t="s">
+      <c r="Z10" s="2" t="s">
         <v>3790</v>
-      </c>
-      <c r="Z10" s="2" t="s">
-        <v>3791</v>
       </c>
       <c r="AF10" s="2">
         <v>10</v>
@@ -13532,17 +13541,20 @@
       </c>
     </row>
     <row r="11" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>101514</v>
+      </c>
       <c r="B11" s="2" t="s">
+        <v>3802</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>3803</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>3804</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>3805</v>
-      </c>
       <c r="J11" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q11" s="2">
         <v>49000</v>
@@ -13551,13 +13563,13 @@
         <v>999</v>
       </c>
       <c r="W11" s="2" t="s">
+        <v>3787</v>
+      </c>
+      <c r="X11" s="2" t="s">
         <v>3788</v>
       </c>
-      <c r="X11" s="2" t="s">
-        <v>3789</v>
-      </c>
       <c r="Y11" s="2" t="s">
-        <v>3791</v>
+        <v>3790</v>
       </c>
       <c r="AF11" s="2">
         <v>10</v>
@@ -13576,17 +13588,20 @@
       </c>
     </row>
     <row r="12" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>101514</v>
+      </c>
       <c r="B12" s="2" t="s">
+        <v>3805</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>3806</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>3807</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>3808</v>
-      </c>
       <c r="J12" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q12" s="2">
         <v>49000</v>
@@ -13595,13 +13610,13 @@
         <v>999</v>
       </c>
       <c r="W12" s="2" t="s">
+        <v>3787</v>
+      </c>
+      <c r="X12" s="2" t="s">
         <v>3788</v>
       </c>
-      <c r="X12" s="2" t="s">
-        <v>3789</v>
-      </c>
       <c r="Y12" s="2" t="s">
-        <v>3791</v>
+        <v>3790</v>
       </c>
       <c r="AF12" s="2">
         <v>10</v>
@@ -13620,17 +13635,20 @@
       </c>
     </row>
     <row r="13" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>101514</v>
+      </c>
       <c r="B13" s="2" t="s">
+        <v>3808</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>3809</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="I13" s="2" t="s">
         <v>3810</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>3811</v>
-      </c>
       <c r="J13" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q13" s="2">
         <v>49000</v>
@@ -13639,13 +13657,13 @@
         <v>999</v>
       </c>
       <c r="W13" s="2" t="s">
-        <v>3792</v>
+        <v>3791</v>
       </c>
       <c r="X13" s="2" t="s">
-        <v>3789</v>
+        <v>3788</v>
       </c>
       <c r="Y13" s="2" t="s">
-        <v>3791</v>
+        <v>3790</v>
       </c>
       <c r="AF13" s="2">
         <v>10</v>
@@ -13664,17 +13682,20 @@
       </c>
     </row>
     <row r="14" spans="1:38" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>101514</v>
+      </c>
       <c r="B14" s="2" t="s">
+        <v>3811</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>3812</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="I14" s="2" t="s">
         <v>3813</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>3814</v>
-      </c>
       <c r="J14" s="2" t="s">
-        <v>3787</v>
+        <v>165</v>
       </c>
       <c r="Q14" s="2">
         <v>99000</v>
@@ -13683,13 +13704,13 @@
         <v>999</v>
       </c>
       <c r="W14" s="2" t="s">
+        <v>3787</v>
+      </c>
+      <c r="X14" s="2" t="s">
+        <v>3790</v>
+      </c>
+      <c r="Y14" s="2" t="s">
         <v>3788</v>
-      </c>
-      <c r="X14" s="2" t="s">
-        <v>3791</v>
-      </c>
-      <c r="Y14" s="2" t="s">
-        <v>3789</v>
       </c>
       <c r="AF14" s="2">
         <v>10</v>

</xml_diff>